<commit_message>
Entrega final 14/10: robo revisado, 383 precos
</commit_message>
<xml_diff>
--- a/FNDE/Centro Oeste/Entrega/dashboard_resumo_coleta.xlsx
+++ b/FNDE/Centro Oeste/Entrega/dashboard_resumo_coleta.xlsx
@@ -2539,10 +2539,10 @@
         </is>
       </c>
       <c r="D2" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" s="15" t="n">
         <v>2</v>
-      </c>
-      <c r="E2" s="15" t="n">
-        <v>3</v>
       </c>
       <c r="F2" s="15">
         <f>D2+E2</f>
@@ -2761,10 +2761,10 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" s="15">
         <f>D8+E8</f>
@@ -2835,10 +2835,10 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" s="15">
         <f>D10+E10</f>
@@ -2872,10 +2872,10 @@
         </is>
       </c>
       <c r="D11" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" s="15">
         <f>D11+E11</f>
@@ -2909,10 +2909,10 @@
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F12" s="15">
         <f>D12+E12</f>
@@ -3020,10 +3020,10 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F15" s="15">
         <f>D15+E15</f>
@@ -3205,10 +3205,10 @@
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" s="15">
         <f>D20+E20</f>
@@ -3427,10 +3427,10 @@
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" s="15">
         <f>D26+E26</f>
@@ -3686,10 +3686,10 @@
         </is>
       </c>
       <c r="D33" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E33" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F33" s="15">
         <f>D33+E33</f>
@@ -3797,10 +3797,10 @@
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F36" s="15">
         <f>D36+E36</f>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="H36" s="15" t="n"/>
       <c r="I36" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J36" s="15">
         <f>IF(E36=0,"Completo",IF(D36=0,"Sem preço","Parcial"))</f>
@@ -4019,10 +4019,10 @@
         </is>
       </c>
       <c r="D42" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" s="15" t="n">
         <v>2</v>
-      </c>
-      <c r="E42" s="15" t="n">
-        <v>3</v>
       </c>
       <c r="F42" s="15">
         <f>D42+E42</f>
@@ -4167,10 +4167,10 @@
         </is>
       </c>
       <c r="D46" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F46" s="15">
         <f>D46+E46</f>
@@ -4463,10 +4463,10 @@
         </is>
       </c>
       <c r="D54" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E54" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F54" s="15">
         <f>D54+E54</f>
@@ -4537,10 +4537,10 @@
         </is>
       </c>
       <c r="D56" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F56" s="15">
         <f>D56+E56</f>
@@ -4722,10 +4722,10 @@
         </is>
       </c>
       <c r="D61" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E61" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F61" s="15">
         <f>D61+E61</f>
@@ -4833,10 +4833,10 @@
         </is>
       </c>
       <c r="D64" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E64" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" s="15">
         <f>D64+E64</f>
@@ -4907,10 +4907,10 @@
         </is>
       </c>
       <c r="D66" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E66" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F66" s="15">
         <f>D66+E66</f>
@@ -5018,10 +5018,10 @@
         </is>
       </c>
       <c r="D69" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E69" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F69" s="15">
         <f>D69+E69</f>
@@ -5721,10 +5721,10 @@
         </is>
       </c>
       <c r="D88" s="15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E88" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F88" s="15">
         <f>D88+E88</f>
@@ -5795,10 +5795,10 @@
         </is>
       </c>
       <c r="D90" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E90" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F90" s="15">
         <f>D90+E90</f>
@@ -5943,10 +5943,10 @@
         </is>
       </c>
       <c r="D94" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E94" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F94" s="15">
         <f>D94+E94</f>
@@ -6017,10 +6017,10 @@
         </is>
       </c>
       <c r="D96" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E96" s="15" t="n">
         <v>2</v>
-      </c>
-      <c r="E96" s="15" t="n">
-        <v>3</v>
       </c>
       <c r="F96" s="15">
         <f>D96+E96</f>
@@ -6202,10 +6202,10 @@
         </is>
       </c>
       <c r="D101" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E101" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F101" s="15">
         <f>D101+E101</f>
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="D104" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E104" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F104" s="15">
         <f>D104+E104</f>
@@ -6350,10 +6350,10 @@
         </is>
       </c>
       <c r="D105" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E105" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F105" s="15">
         <f>D105+E105</f>
@@ -6572,10 +6572,10 @@
         </is>
       </c>
       <c r="D111" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E111" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F111" s="15">
         <f>D111+E111</f>
@@ -6609,10 +6609,10 @@
         </is>
       </c>
       <c r="D112" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E112" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F112" s="15">
         <f>D112+E112</f>
@@ -6720,10 +6720,10 @@
         </is>
       </c>
       <c r="D115" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E115" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F115" s="15">
         <f>D115+E115</f>
@@ -6757,10 +6757,10 @@
         </is>
       </c>
       <c r="D116" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E116" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F116" s="15">
         <f>D116+E116</f>
@@ -6974,7 +6974,7 @@
     <row r="124">
       <c r="A124" s="22" t="inlineStr">
         <is>
-          <t>• Fonte: resumo_coleta.csv de cada grupo, gerados por scripts/montar_merge.py a partir de fnde_resultado_merge.xlsx (montagem de 13/10/2026 21:30).</t>
+          <t>• Fonte: resumo_coleta.csv de cada grupo, gerados por scripts/montar_merge.py a partir de fnde_resultado_merge.xlsx (montagem de 14/10/2026 11:13).</t>
         </is>
       </c>
     </row>

</xml_diff>